<commit_message>
Data Quality: Stage Gate project type, nightly snapshots, no Record now
Project Type reads Stage Gate Project Type. Daily tracking is built from the 11 PM Eastern copies of the
project file and compares the latest data with the previous day's copy. Setup: docs/DAILY-SNAPSHOT.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/dq-project-fixture.xlsx
+++ b/tests/fixtures/dq-project-fixture.xlsx
@@ -796,6 +796,9 @@
       <c r="N2" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q2" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y2">
         <v>7001000</v>
       </c>
@@ -849,9 +852,6 @@
       </c>
       <c r="DO2" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP2" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ2" t="str">
         <v>R-004</v>
@@ -888,6 +888,9 @@
       <c r="N3" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q3" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y3">
         <v>7002000</v>
       </c>
@@ -941,9 +944,6 @@
       </c>
       <c r="DO3" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP3" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ3" t="str">
         <v>R-002</v>
@@ -980,6 +980,9 @@
       <c r="N4" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q4" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y4">
         <v>7003000</v>
       </c>
@@ -1033,9 +1036,6 @@
       </c>
       <c r="DO4" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP4" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ4" t="str">
         <v>R-004</v>
@@ -1072,6 +1072,9 @@
       <c r="N5" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q5" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y5">
         <v>7004000</v>
       </c>
@@ -1125,9 +1128,6 @@
       </c>
       <c r="DO5" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP5" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ5" t="str">
         <v>R-003</v>
@@ -1164,6 +1164,9 @@
       <c r="N6" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q6" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y6">
         <v>7005000</v>
       </c>
@@ -1214,9 +1217,6 @@
       </c>
       <c r="DO6" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP6" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ6" t="str">
         <v>R-002</v>
@@ -1253,6 +1253,9 @@
       <c r="N7" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q7" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y7">
         <v>7006000</v>
       </c>
@@ -1303,9 +1306,6 @@
       </c>
       <c r="DO7" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP7" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ7" t="str">
         <v>R-005</v>
@@ -1342,6 +1342,9 @@
       <c r="N8" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q8" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y8">
         <v>7007000</v>
       </c>
@@ -1395,9 +1398,6 @@
       </c>
       <c r="DO8" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP8" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ8" t="str">
         <v>R-001</v>
@@ -1434,6 +1434,9 @@
       <c r="N9" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q9" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y9">
         <v>7008000</v>
       </c>
@@ -1472,9 +1475,6 @@
       </c>
       <c r="DO9" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP9" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ9" t="str">
         <v>R-004</v>
@@ -1511,6 +1511,9 @@
       <c r="N10" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q10" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y10">
         <v>7009000</v>
       </c>
@@ -1555,9 +1558,6 @@
       </c>
       <c r="DO10" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP10" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ10" t="str">
         <v>R-002</v>
@@ -1594,6 +1594,9 @@
       <c r="N11" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q11" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y11">
         <v>7010000</v>
       </c>
@@ -1641,9 +1644,6 @@
       </c>
       <c r="DO11" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP11" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ11" t="str">
         <v>R-004</v>
@@ -1680,6 +1680,9 @@
       <c r="N12" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q12" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y12">
         <v>7011000</v>
       </c>
@@ -1727,9 +1730,6 @@
       </c>
       <c r="DO12" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP12" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ12" t="str">
         <v>R-004</v>
@@ -1766,6 +1766,9 @@
       <c r="N13" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q13" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y13">
         <v>7012000</v>
       </c>
@@ -1816,9 +1819,6 @@
       </c>
       <c r="DO13" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP13" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ13" t="str">
         <v>R-001</v>
@@ -1855,6 +1855,9 @@
       <c r="N14" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q14" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y14">
         <v>7013000</v>
       </c>
@@ -1908,9 +1911,6 @@
       </c>
       <c r="DO14" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP14" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ14" t="str">
         <v>R-005</v>
@@ -1947,6 +1947,9 @@
       <c r="N15" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q15" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y15">
         <v>7014000</v>
       </c>
@@ -2000,9 +2003,6 @@
       </c>
       <c r="DO15" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP15" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ15" t="str">
         <v>R-001</v>
@@ -2039,6 +2039,9 @@
       <c r="N16" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q16" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y16">
         <v>7015000</v>
       </c>
@@ -2089,9 +2092,6 @@
       </c>
       <c r="DO16" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP16" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ16" t="str">
         <v>R-005</v>
@@ -2128,6 +2128,9 @@
       <c r="N17" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q17" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y17">
         <v>7016000</v>
       </c>
@@ -2181,9 +2184,6 @@
       </c>
       <c r="DO17" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP17" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ17" t="str">
         <v>R-004</v>
@@ -2217,6 +2217,9 @@
       <c r="K18" t="str">
         <v>Tanaka, Eli</v>
       </c>
+      <c r="Q18" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y18">
         <v>7017000</v>
       </c>
@@ -2270,9 +2273,6 @@
       </c>
       <c r="DO18" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP18" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ18" t="str">
         <v>R-005</v>
@@ -2309,6 +2309,9 @@
       <c r="N19" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q19" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y19">
         <v>7018000</v>
       </c>
@@ -2362,9 +2365,6 @@
       </c>
       <c r="DO19" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP19" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ19" t="str">
         <v>R-007</v>
@@ -2401,6 +2401,9 @@
       <c r="N20" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q20" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y20">
         <v>7019000</v>
       </c>
@@ -2454,9 +2457,6 @@
       </c>
       <c r="DO20" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP20" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ20" t="str">
         <v>R-003</v>
@@ -2493,6 +2493,9 @@
       <c r="N21" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q21" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y21">
         <v>7020000</v>
       </c>
@@ -2546,9 +2549,6 @@
       </c>
       <c r="DO21" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP21" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ21" t="str">
         <v>R-004</v>
@@ -2585,6 +2585,9 @@
       <c r="N22" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q22" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y22">
         <v>7021000</v>
       </c>
@@ -2638,9 +2641,6 @@
       </c>
       <c r="DO22" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP22" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ22" t="str">
         <v>R-005</v>
@@ -2677,6 +2677,9 @@
       <c r="N23" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q23" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y23">
         <v>7022000</v>
       </c>
@@ -2715,9 +2718,6 @@
       </c>
       <c r="DO23" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP23" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ23" t="str">
         <v>R-004</v>
@@ -2754,6 +2754,9 @@
       <c r="N24" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q24" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y24">
         <v>7023000</v>
       </c>
@@ -2792,9 +2795,6 @@
       </c>
       <c r="DO24" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP24" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ24" t="str">
         <v>R-004</v>
@@ -2831,6 +2831,9 @@
       <c r="N25" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q25" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y25">
         <v>7024000</v>
       </c>
@@ -2884,9 +2887,6 @@
       </c>
       <c r="DO25" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP25" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ25" t="str">
         <v>R-004</v>
@@ -2923,6 +2923,9 @@
       <c r="N26" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q26" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y26">
         <v>7025000</v>
       </c>
@@ -2976,9 +2979,6 @@
       </c>
       <c r="DO26" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP26" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ26" t="str">
         <v>R-001</v>
@@ -3015,6 +3015,9 @@
       <c r="N27" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q27" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y27">
         <v>7026000</v>
       </c>
@@ -3068,9 +3071,6 @@
       </c>
       <c r="DO27" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP27" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ27" t="str">
         <v>R-001</v>
@@ -3107,6 +3107,9 @@
       <c r="N28" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q28" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y28">
         <v>7027000</v>
       </c>
@@ -3160,9 +3163,6 @@
       </c>
       <c r="DO28" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP28" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ28" t="str">
         <v>R-003</v>
@@ -3199,6 +3199,9 @@
       <c r="N29" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q29" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y29">
         <v>7028000</v>
       </c>
@@ -3252,9 +3255,6 @@
       </c>
       <c r="DO29" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP29" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ29" t="str">
         <v>R-001</v>
@@ -3291,6 +3291,9 @@
       <c r="N30" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q30" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y30">
         <v>7029000</v>
       </c>
@@ -3344,9 +3347,6 @@
       </c>
       <c r="DO30" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP30" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ30" t="str">
         <v>R-001</v>
@@ -3383,6 +3383,9 @@
       <c r="N31" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q31" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y31">
         <v>7030000</v>
       </c>
@@ -3436,9 +3439,6 @@
       </c>
       <c r="DO31" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP31" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ31" t="str">
         <v>R-001</v>
@@ -3475,6 +3475,9 @@
       <c r="N32" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q32" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y32">
         <v>7031000</v>
       </c>
@@ -3528,9 +3531,6 @@
       </c>
       <c r="DO32" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP32" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ32" t="str">
         <v>R-003</v>
@@ -3567,6 +3567,9 @@
       <c r="N33" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q33" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y33">
         <v>7032000</v>
       </c>
@@ -3620,9 +3623,6 @@
       </c>
       <c r="DO33" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP33" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ33" t="str">
         <v>R-002</v>
@@ -3659,6 +3659,9 @@
       <c r="N34" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q34" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y34">
         <v>7033000</v>
       </c>
@@ -3706,9 +3709,6 @@
       </c>
       <c r="DO34" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP34" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ34" t="str">
         <v>R-005</v>
@@ -3745,6 +3745,9 @@
       <c r="N35" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q35" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y35">
         <v>7034000</v>
       </c>
@@ -3792,9 +3795,6 @@
       </c>
       <c r="DO35" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP35" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ35" t="str">
         <v>R-002</v>
@@ -3831,6 +3831,9 @@
       <c r="N36" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q36" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y36">
         <v>7035000</v>
       </c>
@@ -3884,9 +3887,6 @@
       </c>
       <c r="DO36" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP36" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ36" t="str">
         <v>R-004</v>
@@ -3923,6 +3923,9 @@
       <c r="N37" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q37" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y37">
         <v>7036000</v>
       </c>
@@ -3970,9 +3973,6 @@
       </c>
       <c r="DO37" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP37" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ37" t="str">
         <v>R-001</v>
@@ -4009,6 +4009,9 @@
       <c r="N38" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q38" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y38">
         <v>7037000</v>
       </c>
@@ -4056,9 +4059,6 @@
       </c>
       <c r="DO38" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP38" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ38" t="str">
         <v>R-005</v>
@@ -4095,6 +4095,9 @@
       <c r="N39" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q39" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y39">
         <v>7038000</v>
       </c>
@@ -4148,9 +4151,6 @@
       </c>
       <c r="DO39" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP39" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ39" t="str">
         <v>R-004</v>
@@ -4187,6 +4187,9 @@
       <c r="N40" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q40" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y40">
         <v>7039000</v>
       </c>
@@ -4240,9 +4243,6 @@
       </c>
       <c r="DO40" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP40" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ40" t="str">
         <v>R-004</v>
@@ -4279,6 +4279,9 @@
       <c r="N41" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q41" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y41">
         <v>7040000</v>
       </c>
@@ -4332,9 +4335,6 @@
       </c>
       <c r="DO41" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP41" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ41" t="str">
         <v>R-005</v>
@@ -4371,6 +4371,9 @@
       <c r="N42" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q42" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y42">
         <v>7041000</v>
       </c>
@@ -4424,9 +4427,6 @@
       </c>
       <c r="DO42" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP42" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ42" t="str">
         <v>R-005</v>
@@ -4463,6 +4463,9 @@
       <c r="N43" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q43" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y43">
         <v>7042000</v>
       </c>
@@ -4510,9 +4513,6 @@
       </c>
       <c r="DO43" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP43" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ43" t="str">
         <v>R-004</v>
@@ -4549,6 +4549,9 @@
       <c r="N44" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q44" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y44">
         <v>7043000</v>
       </c>
@@ -4596,9 +4599,6 @@
       </c>
       <c r="DO44" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP44" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ44" t="str">
         <v>R-005</v>
@@ -4635,6 +4635,9 @@
       <c r="N45" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q45" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y45">
         <v>7044000</v>
       </c>
@@ -4688,9 +4691,6 @@
       </c>
       <c r="DO45" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP45" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ45" t="str">
         <v>R-004</v>
@@ -4727,6 +4727,9 @@
       <c r="N46" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q46" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y46">
         <v>7045000</v>
       </c>
@@ -4780,9 +4783,6 @@
       </c>
       <c r="DO46" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP46" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ46" t="str">
         <v>R-005</v>
@@ -4819,6 +4819,9 @@
       <c r="N47" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q47" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y47">
         <v>7046000</v>
       </c>
@@ -4872,9 +4875,6 @@
       </c>
       <c r="DO47" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP47" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ47" t="str">
         <v>R-005</v>
@@ -4911,6 +4911,9 @@
       <c r="N48" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q48" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y48">
         <v>7047000</v>
       </c>
@@ -4964,9 +4967,6 @@
       </c>
       <c r="DO48" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP48" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ48" t="str">
         <v>R-004</v>
@@ -5003,6 +5003,9 @@
       <c r="N49" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q49" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y49">
         <v>7048000</v>
       </c>
@@ -5056,9 +5059,6 @@
       </c>
       <c r="DO49" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP49" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ49" t="str">
         <v>R-005</v>
@@ -5095,6 +5095,9 @@
       <c r="N50" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q50" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y50">
         <v>7049000</v>
       </c>
@@ -5142,9 +5145,6 @@
       </c>
       <c r="DO50" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP50" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ50" t="str">
         <v>R-005</v>
@@ -5181,6 +5181,9 @@
       <c r="N51" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q51" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y51">
         <v>7050000</v>
       </c>
@@ -5228,9 +5231,6 @@
       </c>
       <c r="DO51" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP51" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ51" t="str">
         <v>R-005</v>
@@ -5267,6 +5267,9 @@
       <c r="N52" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q52" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y52">
         <v>7051000</v>
       </c>
@@ -5320,9 +5323,6 @@
       </c>
       <c r="DO52" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP52" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ52" t="str">
         <v>R-005</v>
@@ -5359,6 +5359,9 @@
       <c r="N53" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q53" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y53">
         <v>7052000</v>
       </c>
@@ -5412,9 +5415,6 @@
       </c>
       <c r="DO53" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP53" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ53" t="str">
         <v>R-004</v>
@@ -5451,6 +5451,9 @@
       <c r="N54" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q54" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y54">
         <v>7053000</v>
       </c>
@@ -5504,9 +5507,6 @@
       </c>
       <c r="DO54" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP54" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ54" t="str">
         <v>R-004</v>
@@ -5543,6 +5543,9 @@
       <c r="N55" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q55" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y55">
         <v>7054000</v>
       </c>
@@ -5596,9 +5599,6 @@
       </c>
       <c r="DO55" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP55" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ55" t="str">
         <v>R-004</v>
@@ -5635,6 +5635,9 @@
       <c r="N56" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q56" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y56">
         <v>7055000</v>
       </c>
@@ -5688,9 +5691,6 @@
       </c>
       <c r="DO56" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP56" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ56" t="str">
         <v>R-001</v>
@@ -5727,6 +5727,9 @@
       <c r="N57" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q57" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y57">
         <v>7056000</v>
       </c>
@@ -5780,9 +5783,6 @@
       </c>
       <c r="DO57" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP57" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ57" t="str">
         <v>R-001</v>
@@ -5819,6 +5819,9 @@
       <c r="N58" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q58" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y58">
         <v>7057000</v>
       </c>
@@ -5872,9 +5875,6 @@
       </c>
       <c r="DO58" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP58" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ58" t="str">
         <v>R-002</v>
@@ -5911,6 +5911,9 @@
       <c r="N59" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q59" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y59">
         <v>7058000</v>
       </c>
@@ -5964,9 +5967,6 @@
       </c>
       <c r="DO59" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP59" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ59" t="str">
         <v>R-001</v>
@@ -6003,6 +6003,9 @@
       <c r="N60" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q60" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y60">
         <v>7059000</v>
       </c>
@@ -6056,9 +6059,6 @@
       </c>
       <c r="DO60" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP60" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ60" t="str">
         <v>R-004</v>
@@ -6095,6 +6095,9 @@
       <c r="N61" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q61" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y61">
         <v>7060000</v>
       </c>
@@ -6148,9 +6151,6 @@
       </c>
       <c r="DO61" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP61" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ61" t="str">
         <v>R-005</v>
@@ -6187,6 +6187,9 @@
       <c r="N62" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q62" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y62">
         <v>7061000</v>
       </c>
@@ -6240,9 +6243,6 @@
       </c>
       <c r="DO62" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP62" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ62" t="str">
         <v>R-004</v>
@@ -6279,6 +6279,9 @@
       <c r="N63" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q63" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y63">
         <v>7062000</v>
       </c>
@@ -6332,9 +6335,6 @@
       </c>
       <c r="DO63" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP63" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ63" t="str">
         <v>R-004</v>
@@ -6371,6 +6371,9 @@
       <c r="N64" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q64" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y64">
         <v>7063000</v>
       </c>
@@ -6424,9 +6427,6 @@
       </c>
       <c r="DO64" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP64" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ64" t="str">
         <v>R-002</v>
@@ -6463,6 +6463,9 @@
       <c r="N65" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q65" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y65">
         <v>7064000</v>
       </c>
@@ -6516,9 +6519,6 @@
       </c>
       <c r="DO65" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP65" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ65" t="str">
         <v>R-003</v>
@@ -6555,6 +6555,9 @@
       <c r="N66" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q66" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y66">
         <v>7065000</v>
       </c>
@@ -6608,9 +6611,6 @@
       </c>
       <c r="DO66" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP66" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ66" t="str">
         <v>R-003</v>
@@ -6647,6 +6647,9 @@
       <c r="N67" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q67" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y67">
         <v>7066000</v>
       </c>
@@ -6700,9 +6703,6 @@
       </c>
       <c r="DO67" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP67" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ67" t="str">
         <v>R-004</v>
@@ -6739,6 +6739,9 @@
       <c r="N68" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q68" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y68">
         <v>7067000</v>
       </c>
@@ -6792,9 +6795,6 @@
       </c>
       <c r="DO68" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP68" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ68" t="str">
         <v>R-001</v>
@@ -6831,6 +6831,9 @@
       <c r="N69" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q69" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y69">
         <v>7068000</v>
       </c>
@@ -6884,9 +6887,6 @@
       </c>
       <c r="DO69" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP69" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ69" t="str">
         <v>R-001</v>
@@ -6923,6 +6923,9 @@
       <c r="N70" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q70" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y70">
         <v>7069000</v>
       </c>
@@ -6976,9 +6979,6 @@
       </c>
       <c r="DO70" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP70" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ70" t="str">
         <v>R-005</v>
@@ -7015,6 +7015,9 @@
       <c r="N71" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q71" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y71">
         <v>7070000</v>
       </c>
@@ -7068,9 +7071,6 @@
       </c>
       <c r="DO71" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP71" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ71" t="str">
         <v>R-004</v>
@@ -7107,6 +7107,9 @@
       <c r="N72" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q72" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y72">
         <v>7071000</v>
       </c>
@@ -7154,9 +7157,6 @@
       </c>
       <c r="DO72" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP72" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ72" t="str">
         <v>R-004</v>
@@ -7193,6 +7193,9 @@
       <c r="N73" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q73" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y73">
         <v>7072000</v>
       </c>
@@ -7246,9 +7249,6 @@
       </c>
       <c r="DO73" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP73" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ73" t="str">
         <v>R-002</v>
@@ -7285,6 +7285,9 @@
       <c r="N74" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q74" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y74">
         <v>7073000</v>
       </c>
@@ -7338,9 +7341,6 @@
       </c>
       <c r="DO74" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP74" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ74" t="str">
         <v>R-001</v>
@@ -7377,6 +7377,9 @@
       <c r="N75" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q75" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y75">
         <v>7074000</v>
       </c>
@@ -7430,9 +7433,6 @@
       </c>
       <c r="DO75" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP75" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ75" t="str">
         <v>R-003</v>
@@ -7469,6 +7469,9 @@
       <c r="N76" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q76" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y76">
         <v>7075000</v>
       </c>
@@ -7516,9 +7519,6 @@
       </c>
       <c r="DO76" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP76" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ76" t="str">
         <v>R-005</v>
@@ -7555,6 +7555,9 @@
       <c r="N77" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q77" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y77">
         <v>7076000</v>
       </c>
@@ -7608,9 +7611,6 @@
       </c>
       <c r="DO77" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP77" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ77" t="str">
         <v>R-002</v>
@@ -7647,6 +7647,9 @@
       <c r="N78" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q78" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y78">
         <v>7077000</v>
       </c>
@@ -7694,9 +7697,6 @@
       </c>
       <c r="DO78" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP78" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ78" t="str">
         <v>R-005</v>
@@ -7733,6 +7733,9 @@
       <c r="N79" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q79" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y79">
         <v>7078000</v>
       </c>
@@ -7786,9 +7789,6 @@
       </c>
       <c r="DO79" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP79" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ79" t="str">
         <v>R-005</v>
@@ -7825,6 +7825,9 @@
       <c r="N80" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q80" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y80">
         <v>7079000</v>
       </c>
@@ -7878,9 +7881,6 @@
       </c>
       <c r="DO80" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP80" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ80" t="str">
         <v>R-005</v>
@@ -7917,6 +7917,9 @@
       <c r="N81" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q81" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y81">
         <v>7080000</v>
       </c>
@@ -7970,9 +7973,6 @@
       </c>
       <c r="DO81" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP81" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ81" t="str">
         <v>R-002</v>
@@ -8009,6 +8009,9 @@
       <c r="N82" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q82" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y82">
         <v>7081000</v>
       </c>
@@ -8062,9 +8065,6 @@
       </c>
       <c r="DO82" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP82" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ82" t="str">
         <v>R-001</v>
@@ -8101,6 +8101,9 @@
       <c r="N83" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q83" t="str">
+        <v>Improvement.On Platform</v>
+      </c>
       <c r="Y83">
         <v>7082000</v>
       </c>
@@ -8148,9 +8151,6 @@
       </c>
       <c r="DO83" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP83" t="str">
-        <v>Improvement.On Platform</v>
       </c>
       <c r="DQ83" t="str">
         <v>R-003</v>
@@ -8187,6 +8187,9 @@
       <c r="N84" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q84" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y84">
         <v>7083000</v>
       </c>
@@ -8240,9 +8243,6 @@
       </c>
       <c r="DO84" s="1">
         <v>46482</v>
-      </c>
-      <c r="DP84" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ84" t="str">
         <v>R-003</v>
@@ -8279,6 +8279,9 @@
       <c r="N85" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q85" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y85">
         <v>7084000</v>
       </c>
@@ -8332,9 +8335,6 @@
       </c>
       <c r="DO85" s="1">
         <v>46512</v>
-      </c>
-      <c r="DP85" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ85" t="str">
         <v>R-001</v>
@@ -8371,6 +8371,9 @@
       <c r="N86" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q86" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y86">
         <v>7085000</v>
       </c>
@@ -8424,9 +8427,6 @@
       </c>
       <c r="DO86" s="1">
         <v>46543</v>
-      </c>
-      <c r="DP86" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ86" t="str">
         <v>R-004</v>
@@ -8463,6 +8463,9 @@
       <c r="N87" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q87" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y87">
         <v>7086000</v>
       </c>
@@ -8516,9 +8519,6 @@
       </c>
       <c r="DO87" s="1">
         <v>46573</v>
-      </c>
-      <c r="DP87" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ87" t="str">
         <v>R-003</v>
@@ -8555,6 +8555,9 @@
       <c r="N88" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q88" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y88">
         <v>7087000</v>
       </c>
@@ -8608,9 +8611,6 @@
       </c>
       <c r="DO88" s="1">
         <v>46604</v>
-      </c>
-      <c r="DP88" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ88" t="str">
         <v>R-004</v>
@@ -8647,6 +8647,9 @@
       <c r="N89" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q89" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y89">
         <v>7088000</v>
       </c>
@@ -8700,9 +8703,6 @@
       </c>
       <c r="DO89" s="1">
         <v>46635</v>
-      </c>
-      <c r="DP89" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ89" t="str">
         <v>R-005</v>
@@ -8739,6 +8739,9 @@
       <c r="N90" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q90" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y90">
         <v>7089000</v>
       </c>
@@ -8792,9 +8795,6 @@
       </c>
       <c r="DO90" s="1">
         <v>46665</v>
-      </c>
-      <c r="DP90" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ90" t="str">
         <v>R-002</v>
@@ -8831,6 +8831,9 @@
       <c r="N91" t="str">
         <v>Alpha</v>
       </c>
+      <c r="Q91" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y91">
         <v>7090000</v>
       </c>
@@ -8884,9 +8887,6 @@
       </c>
       <c r="DO91" s="1">
         <v>46696</v>
-      </c>
-      <c r="DP91" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ91" t="str">
         <v>R-005</v>
@@ -8923,6 +8923,9 @@
       <c r="N92" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q92" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y92">
         <v>7091000</v>
       </c>
@@ -8976,9 +8979,6 @@
       </c>
       <c r="DO92" s="1">
         <v>46726</v>
-      </c>
-      <c r="DP92" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ92" t="str">
         <v>R-005</v>
@@ -9015,6 +9015,9 @@
       <c r="N93" t="str">
         <v>Gamma</v>
       </c>
+      <c r="Q93" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y93">
         <v>7092000</v>
       </c>
@@ -9068,9 +9071,6 @@
       </c>
       <c r="DO93" s="1">
         <v>46392</v>
-      </c>
-      <c r="DP93" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ93" t="str">
         <v>R-002</v>
@@ -9107,6 +9107,9 @@
       <c r="N94" t="str">
         <v>Beta</v>
       </c>
+      <c r="Q94" t="str">
+        <v>Compliance.On Platform</v>
+      </c>
       <c r="Y94">
         <v>7093000</v>
       </c>
@@ -9160,9 +9163,6 @@
       </c>
       <c r="DO94" s="1">
         <v>46423</v>
-      </c>
-      <c r="DP94" t="str">
-        <v>Compliance.On Platform</v>
       </c>
       <c r="DQ94" t="str">
         <v>R-003</v>
@@ -9199,6 +9199,9 @@
       <c r="N95" t="str">
         <v>Delta</v>
       </c>
+      <c r="Q95" t="str">
+        <v>Product Expansion/Refresh.On Platform</v>
+      </c>
       <c r="Y95">
         <v>7094000</v>
       </c>
@@ -9252,9 +9255,6 @@
       </c>
       <c r="DO95" s="1">
         <v>46451</v>
-      </c>
-      <c r="DP95" t="str">
-        <v>Product Expansion/Refresh.On Platform</v>
       </c>
       <c r="DQ95" t="str">
         <v>R-005</v>

</xml_diff>